<commit_message>
feat(kpis.py): Se traslada la lógica de las kpis de ventas a kpis.py
</commit_message>
<xml_diff>
--- a/data/estad_portales/Rendimiento_p1.xlsx
+++ b/data/estad_portales/Rendimiento_p1.xlsx
@@ -427,25 +427,25 @@
     </row>
     <row r="2" ht="17" customHeight="1">
       <c r="A2" s="2" t="str">
-        <v>14/08/2026</v>
+        <v>21/08/2026</v>
       </c>
       <c r="B2" s="2">
-        <v>15408</v>
+        <v>18947</v>
       </c>
       <c r="C2" s="2">
-        <v>652</v>
+        <v>900</v>
       </c>
       <c r="D2" s="2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E2" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2" s="2">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G2" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" s="2" t="str">
         <v/>
@@ -453,25 +453,25 @@
     </row>
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="2" t="str">
-        <v>15/08/2026</v>
+        <v>22/08/2026</v>
       </c>
       <c r="B3" s="2">
-        <v>14948</v>
+        <v>21228</v>
       </c>
       <c r="C3" s="2">
-        <v>614</v>
+        <v>779</v>
       </c>
       <c r="D3" s="2">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E3" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="2" t="str">
         <v/>
@@ -479,25 +479,25 @@
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="2" t="str">
-        <v>16/08/2026</v>
+        <v>23/08/2026</v>
       </c>
       <c r="B4" s="2">
-        <v>16586</v>
+        <v>21905</v>
       </c>
       <c r="C4" s="2">
-        <v>574</v>
+        <v>966</v>
       </c>
       <c r="D4" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="str">
         <v/>
@@ -505,25 +505,25 @@
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="2" t="str">
-        <v>17/08/2026</v>
+        <v>24/08/2026</v>
       </c>
       <c r="B5" s="2">
-        <v>18724</v>
+        <v>23098</v>
       </c>
       <c r="C5" s="2">
-        <v>840</v>
+        <v>1056</v>
       </c>
       <c r="D5" s="2">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E5" s="2">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F5" s="2">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G5" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H5" s="2" t="str">
         <v/>
@@ -531,25 +531,25 @@
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="2" t="str">
-        <v>18/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="B6" s="2">
-        <v>19429</v>
+        <v>20750</v>
       </c>
       <c r="C6" s="2">
-        <v>888</v>
+        <v>1028</v>
       </c>
       <c r="D6" s="2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E6" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F6" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G6" s="2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H6" s="2" t="str">
         <v/>
@@ -557,25 +557,25 @@
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="2" t="str">
-        <v>19/08/2026</v>
+        <v>26/08/2026</v>
       </c>
       <c r="B7" s="2">
-        <v>20356</v>
+        <v>19921</v>
       </c>
       <c r="C7" s="2">
-        <v>975</v>
+        <v>918</v>
       </c>
       <c r="D7" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E7" s="2">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" s="2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G7" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H7" s="2" t="str">
         <v/>
@@ -583,25 +583,25 @@
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="2" t="str">
-        <v>20/08/2026</v>
+        <v>27/08/2026</v>
       </c>
       <c r="B8" s="2">
-        <v>20577</v>
+        <v>20561</v>
       </c>
       <c r="C8" s="2">
-        <v>907</v>
+        <v>899</v>
       </c>
       <c r="D8" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E8" s="2">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2">
         <v>10</v>
       </c>
-      <c r="F8" s="2">
-        <v>7</v>
-      </c>
       <c r="G8" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8" s="2" t="str">
         <v/>

</xml_diff>